<commit_message>
Rebuild attribution reference on Windows
</commit_message>
<xml_diff>
--- a/artifacts/任务规格转化.xlsx
+++ b/artifacts/任务规格转化.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R6a17aca9eb7f4f1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="任务规格转化" sheetId="1" r:id="R1d24788abd9746ed"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -453,22 +453,6 @@
         <x:v>PowerShell入口返回0，数据库、SQL和三张CSV可读，派生表与报表一致</x:v>
       </x:c>
     </x:row>
-    <x:row r="19" ht="33" customHeight="1">
-      <x:c r="A19" s="5" t="str">
-        <x:v>可验证点</x:v>
-      </x:c>
-      <x:c r="B19" s="5" t="str">
-        <x:v>源表保全、曝光主键、污染原因、转化匹配、窗口状态、分组指标与跨产物对账</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="33" customHeight="1">
-      <x:c r="A20" s="5" t="str">
-        <x:v>不适合作为评分点的内容</x:v>
-      </x:c>
-      <x:c r="B20" s="5" t="str">
-        <x:v>CTE拆分、别名、索引名、注释、缩进、内部查询顺序、CSV必要引号和LF或CRLF行尾</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>